<commit_message>
live update of tasks
</commit_message>
<xml_diff>
--- a/task_reports.xlsx
+++ b/task_reports.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B209"/>
+  <dimension ref="A1:B210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="25" customWidth="1" style="1" min="1" max="1"/>
@@ -3064,7 +3064,9 @@
       <c r="B202" s="3" t="inlineStr">
         <is>
           <t>[ONEX-Academy]
-• make the cards with nice pictures, remove the onex@onex.am thing from the cards, make only ONEX maybe</t>
+• make the cards with nice pictures, remove the onex@onex.am thing from the cards, make only ONEX maybe
+[DealFinder]
+• continue working on the google extention</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3205,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>06/10/2026 17:34:55</t>
+          <t>06/10/2026 20:28:36</t>
         </is>
       </c>
       <c r="B209" s="3" t="inlineStr">
@@ -3215,7 +3217,25 @@
 [cc-kpi-onex]
 • implement the Kristina's tasks.
 [ai-agents-scores]
-• validate the results and tell Anna</t>
+• validate the results and tell Anna
+[cc-kpi-onex]
+• remove աշխատակից/ կարգ writtings from the ui, its too industrial, and not visual friendly.
+  improve the ui visuals of the upper part of the provided screenshot to be in the ui (do it right, and other motivation writtings)
+  add the levels (bronze silver gold ,etc..) nice visual friendly section with percent showing (shown in the new screenshot)
+  select in calendar the range of internship, so after that, the internship should be unchecked and the agent should become normal worker instead of intern. Also there should be editing function which admin can edit and make an internship worker standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>07/10/2026 19:45:36</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>[Blot]
+• add ai partner feature (ai agents that act like partners with user provided rules)</t>
         </is>
       </c>
     </row>

</xml_diff>